<commit_message>
Add TMC Marine Compressor Lube Plus (301020) supplied stock to requisition workbook
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CUnrZB177HUYZdeNmgVGRz
</commit_message>
<xml_diff>
--- a/out/North_Fleet_Lub_Oil_Requisition.xlsx
+++ b/out/North_Fleet_Lub_Oil_Requisition.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="178">
   <si>
     <r>
       <rPr>
@@ -398,6 +398,74 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">1 PAIL – TMC Lube Plus (L)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">← 가정값</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: P/N 301020 </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">공급분</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: 5 PAILS = 94.5 L, 4 PAILS = 75.6 L (</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사용자 제공 </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ 1 PAIL = 18.9 L)</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">No.</t>
   </si>
   <si>
@@ -606,6 +674,40 @@
       </rPr>
       <t xml:space="preserve">확인 필요</t>
     </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">공급분은 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">TMC MARINE COMPRESSOR LUBE PLUS </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">행 참조</t>
+    </r>
   </si>
   <si>
     <r>
@@ -644,7 +746,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(16) – </t>
+      <t xml:space="preserve">(17) – </t>
     </r>
     <r>
       <rPr>
@@ -693,6 +795,53 @@
     <t xml:space="preserve">PRESLIA 68</t>
   </si>
   <si>
+    <t xml:space="preserve">TMC MARINE COMPRESSOR LUBE PLUS (P/N 301020)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이번 공급분</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(Valley 5 / Ocean 5 / Moon 4 PAILS) – </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">재고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(ROB)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 반영</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">VISGA 15</t>
   </si>
   <si>
@@ -1753,41 +1902,54 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(0)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="10"/>
-        <color rgb="FF7F7F7F"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="10"/>
-        <color rgb="FF7F7F7F"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">해당 없음 – 원본에 청구 없는 품목 없음</t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="10"/>
-        <color rgb="FF7F7F7F"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
+      <t xml:space="preserve">(1)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">4 PAILS (75.6 LT)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이번 공급분 → 재고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(ROB) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">반영</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">청구 없음</t>
     </r>
   </si>
   <si>
@@ -1940,6 +2102,9 @@
   </si>
   <si>
     <t xml:space="preserve">ROB 70 Lit. Required for scheduled maintenenace</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 PAILS (94.5 LT)</t>
   </si>
   <si>
     <t xml:space="preserve">NORTH VALLEY – LUB OIL REQUISITION</t>
@@ -2053,7 +2218,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="[=0]\-;[&gt;=1000]#,##0;General"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2150,21 +2315,6 @@
       <name val="WenQuanYi Zen Hei"/>
       <family val="2"/>
     </font>
-    <font>
-      <i val="true"/>
-      <sz val="10"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <i val="true"/>
-      <sz val="10"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="WenQuanYi Zen Hei"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -2247,7 +2397,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2292,6 +2442,10 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2302,14 +2456,6 @@
     </xf>
     <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2338,7 +2484,7 @@
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFBFBFBF"/>
-      <rgbColor rgb="FF7F7F7F"/>
+      <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFEDEDED"/>
@@ -2564,7 +2710,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M47"/>
+  <dimension ref="A1:M48"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -2607,37 +2753,48 @@
         <v>5</v>
       </c>
     </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="5" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G6" s="5"/>
       <c r="H6" s="5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="I6" s="5"/>
       <c r="J6" s="5" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K6" s="5"/>
       <c r="L6" s="5" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2645,35 +2802,35 @@
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="L7" s="5"/>
       <c r="M7" s="5"/>
     </row>
     <row r="8" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
@@ -2693,10 +2850,10 @@
         <v>1</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D9" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B9,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B9))</f>
@@ -2741,10 +2898,10 @@
         <v>2</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D10" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B10,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B10))</f>
@@ -2789,10 +2946,10 @@
         <v>3</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D11" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B11,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B11))</f>
@@ -2837,10 +2994,10 @@
         <v>4</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D12" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B12,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B12))</f>
@@ -2885,10 +3042,10 @@
         <v>5</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D13" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B13,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B13))</f>
@@ -2927,7 +3084,7 @@
         <v>100</v>
       </c>
       <c r="M13" s="8" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2935,10 +3092,10 @@
         <v>6</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D14" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B14,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B14))</f>
@@ -2983,10 +3140,10 @@
         <v>7</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D15" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B15,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B15))</f>
@@ -3031,10 +3188,10 @@
         <v>8</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D16" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B16,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B16))</f>
@@ -3079,10 +3236,10 @@
         <v>9</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D17" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B17,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B17))</f>
@@ -3127,10 +3284,10 @@
         <v>10</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D18" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B18,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B18))</f>
@@ -3175,10 +3332,10 @@
         <v>11</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D19" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B19,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B19))</f>
@@ -3223,10 +3380,10 @@
         <v>12</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D20" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B20,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B20))</f>
@@ -3271,10 +3428,10 @@
         <v>13</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D21" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B21,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B21))</f>
@@ -3319,10 +3476,10 @@
         <v>14</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D22" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B22,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B22))</f>
@@ -3367,10 +3524,10 @@
         <v>15</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D23" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B23,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B23))</f>
@@ -3415,10 +3572,10 @@
         <v>16</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D24" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B24,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B24))</f>
@@ -3463,10 +3620,10 @@
         <v>17</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D25" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B25,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B25))</f>
@@ -3511,10 +3668,10 @@
         <v>18</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D26" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B26,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B26))</f>
@@ -3559,10 +3716,10 @@
         <v>19</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D27" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B27,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B27))</f>
@@ -3601,7 +3758,7 @@
         <v>1.9</v>
       </c>
       <c r="M27" s="8" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3609,10 +3766,10 @@
         <v>20</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D28" s="9" t="n">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B28,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B28))</f>
@@ -3651,18 +3808,18 @@
         <v>111000</v>
       </c>
       <c r="M28" s="8" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="38.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="n">
         <v>21</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D29" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B29,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B29))</f>
@@ -3701,12 +3858,12 @@
         <v>295.6</v>
       </c>
       <c r="M29" s="8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B31" s="6"/>
       <c r="C31" s="6"/>
@@ -3726,10 +3883,10 @@
         <v>1</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D32" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B32,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B32))</f>
@@ -3774,10 +3931,10 @@
         <v>2</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D33" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B33,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B33))</f>
@@ -3822,10 +3979,10 @@
         <v>3</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D34" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B34,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B34))</f>
@@ -3870,10 +4027,10 @@
         <v>4</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D35" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B35,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B35))</f>
@@ -3918,10 +4075,10 @@
         <v>5</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D36" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B36,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B36))</f>
@@ -3966,10 +4123,10 @@
         <v>6</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D37" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B37,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B37))</f>
@@ -4014,10 +4171,10 @@
         <v>7</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D38" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B38,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B38))</f>
@@ -4062,10 +4219,10 @@
         <v>8</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D39" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B39,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B39))</f>
@@ -4110,10 +4267,10 @@
         <v>9</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D40" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B40,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B40))</f>
@@ -4158,10 +4315,10 @@
         <v>10</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D41" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B41,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B41))</f>
@@ -4206,10 +4363,10 @@
         <v>11</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D42" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B42,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B42))</f>
@@ -4254,10 +4411,10 @@
         <v>12</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D43" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B43,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B43))</f>
@@ -4297,15 +4454,15 @@
       </c>
       <c r="M43" s="8"/>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="n">
         <v>13</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D44" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B44,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B44))</f>
@@ -4315,25 +4472,25 @@
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B44,'North Light'!$F$6:$F$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$F$6:$F$38,'North Light'!$B$6:$B$38,$B44))</f>
         <v/>
       </c>
-      <c r="F44" s="9" t="str">
+      <c r="F44" s="9" t="n">
         <f aca="false">IF(COUNTIFS('North Moon'!$B$6:$B$13,$B44,'North Moon'!$E$6:$E$13,"&lt;&gt;")=0,"",SUMIFS('North Moon'!$E$6:$E$13,'North Moon'!$B$6:$B$13,$B44))</f>
-        <v/>
+        <v>75.6</v>
       </c>
       <c r="G44" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Moon'!$B$6:$B$13,$B44,'North Moon'!$F$6:$F$13,"&lt;&gt;")=0,"",SUMIFS('North Moon'!$F$6:$F$13,'North Moon'!$B$6:$B$13,$B44))</f>
         <v/>
       </c>
-      <c r="H44" s="9" t="str">
+      <c r="H44" s="9" t="n">
         <f aca="false">IF(COUNTIFS('North Ocean'!$B$6:$B$17,$B44,'North Ocean'!$E$6:$E$17,"&lt;&gt;")=0,"",SUMIFS('North Ocean'!$E$6:$E$17,'North Ocean'!$B$6:$B$17,$B44))</f>
-        <v/>
+        <v>94.5</v>
       </c>
       <c r="I44" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Ocean'!$B$6:$B$17,$B44,'North Ocean'!$F$6:$F$17,"&lt;&gt;")=0,"",SUMIFS('North Ocean'!$F$6:$F$17,'North Ocean'!$B$6:$B$17,$B44))</f>
         <v/>
       </c>
-      <c r="J44" s="9" t="str">
+      <c r="J44" s="9" t="n">
         <f aca="false">IF(COUNTIFS('North Valley'!$B$6:$B$22,$B44,'North Valley'!$E$6:$E$22,"&lt;&gt;")=0,"",SUMIFS('North Valley'!$E$6:$E$22,'North Valley'!$B$6:$B$22,$B44))</f>
-        <v/>
+        <v>94.5</v>
       </c>
       <c r="K44" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Valley'!$B$6:$B$22,$B44,'North Valley'!$F$6:$F$22,"&lt;&gt;")=0,"",SUMIFS('North Valley'!$F$6:$F$22,'North Valley'!$B$6:$B$22,$B44))</f>
@@ -4343,17 +4500,19 @@
         <f aca="false">SUM(E44,G44,I44,K44)</f>
         <v>0</v>
       </c>
-      <c r="M44" s="8"/>
+      <c r="M44" s="11" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="n">
         <v>14</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D45" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B45,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B45))</f>
@@ -4398,10 +4557,10 @@
         <v>15</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D46" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B46,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B46))</f>
@@ -4446,10 +4605,10 @@
         <v>16</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D47" s="9" t="str">
         <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B47,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B47))</f>
@@ -4488,6 +4647,54 @@
         <v>0</v>
       </c>
       <c r="M47" s="8"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D48" s="9" t="str">
+        <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B48,'North Light'!$E$6:$E$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$E$6:$E$38,'North Light'!$B$6:$B$38,$B48))</f>
+        <v/>
+      </c>
+      <c r="E48" s="9" t="str">
+        <f aca="false">IF(COUNTIFS('North Light'!$B$6:$B$38,$B48,'North Light'!$F$6:$F$38,"&lt;&gt;")=0,"",SUMIFS('North Light'!$F$6:$F$38,'North Light'!$B$6:$B$38,$B48))</f>
+        <v/>
+      </c>
+      <c r="F48" s="9" t="str">
+        <f aca="false">IF(COUNTIFS('North Moon'!$B$6:$B$13,$B48,'North Moon'!$E$6:$E$13,"&lt;&gt;")=0,"",SUMIFS('North Moon'!$E$6:$E$13,'North Moon'!$B$6:$B$13,$B48))</f>
+        <v/>
+      </c>
+      <c r="G48" s="9" t="str">
+        <f aca="false">IF(COUNTIFS('North Moon'!$B$6:$B$13,$B48,'North Moon'!$F$6:$F$13,"&lt;&gt;")=0,"",SUMIFS('North Moon'!$F$6:$F$13,'North Moon'!$B$6:$B$13,$B48))</f>
+        <v/>
+      </c>
+      <c r="H48" s="9" t="str">
+        <f aca="false">IF(COUNTIFS('North Ocean'!$B$6:$B$17,$B48,'North Ocean'!$E$6:$E$17,"&lt;&gt;")=0,"",SUMIFS('North Ocean'!$E$6:$E$17,'North Ocean'!$B$6:$B$17,$B48))</f>
+        <v/>
+      </c>
+      <c r="I48" s="9" t="str">
+        <f aca="false">IF(COUNTIFS('North Ocean'!$B$6:$B$17,$B48,'North Ocean'!$F$6:$F$17,"&lt;&gt;")=0,"",SUMIFS('North Ocean'!$F$6:$F$17,'North Ocean'!$B$6:$B$17,$B48))</f>
+        <v/>
+      </c>
+      <c r="J48" s="9" t="str">
+        <f aca="false">IF(COUNTIFS('North Valley'!$B$6:$B$22,$B48,'North Valley'!$E$6:$E$22,"&lt;&gt;")=0,"",SUMIFS('North Valley'!$E$6:$E$22,'North Valley'!$B$6:$B$22,$B48))</f>
+        <v/>
+      </c>
+      <c r="K48" s="9" t="str">
+        <f aca="false">IF(COUNTIFS('North Valley'!$B$6:$B$22,$B48,'North Valley'!$F$6:$F$22,"&lt;&gt;")=0,"",SUMIFS('North Valley'!$F$6:$F$22,'North Valley'!$B$6:$B$22,$B48))</f>
+        <v/>
+      </c>
+      <c r="L48" s="10" t="n">
+        <f aca="false">SUM(E48,G48,I48,K48)</f>
+        <v>0</v>
+      </c>
+      <c r="M48" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -4532,48 +4739,48 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="11" t="s">
-        <v>63</v>
+      <c r="A2" s="12" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="11" t="s">
-        <v>64</v>
+      <c r="A3" s="12" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="H5" s="5" t="s">
         <v>16</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -4588,24 +4795,24 @@
         <v>1</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="12"/>
+        <v>21</v>
+      </c>
+      <c r="E7" s="13"/>
       <c r="F7" s="9" t="n">
         <f aca="false">8*'통합 청구'!$C$3</f>
         <v>160</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4613,24 +4820,24 @@
         <v>2</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="12"/>
+        <v>21</v>
+      </c>
+      <c r="E8" s="13"/>
       <c r="F8" s="9" t="n">
         <f aca="false">6*'통합 청구'!$C$3</f>
         <v>120</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4638,23 +4845,23 @@
         <v>3</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C9" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="13"/>
+      <c r="F9" s="14" t="n">
+        <v>108</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="H9" s="8" t="s">
         <v>74</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E9" s="12"/>
-      <c r="F9" s="13" t="n">
-        <v>108</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="H9" s="8" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4662,24 +4869,24 @@
         <v>4</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="12"/>
+        <v>21</v>
+      </c>
+      <c r="E10" s="13"/>
       <c r="F10" s="9" t="n">
         <f aca="false">9*'통합 청구'!$C$3</f>
         <v>180</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4687,23 +4894,23 @@
         <v>5</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C11" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="13"/>
+      <c r="F11" s="14" t="n">
+        <v>108</v>
+      </c>
+      <c r="G11" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="D11" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E11" s="12"/>
-      <c r="F11" s="13" t="n">
-        <v>108</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>75</v>
-      </c>
       <c r="H11" s="8" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4711,24 +4918,24 @@
         <v>6</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="12"/>
+        <v>21</v>
+      </c>
+      <c r="E12" s="13"/>
       <c r="F12" s="9" t="n">
         <f aca="false">2*'통합 청구'!$C$3</f>
         <v>40</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4736,23 +4943,23 @@
         <v>7</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="12"/>
-      <c r="F13" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E13" s="13"/>
+      <c r="F13" s="14" t="n">
         <v>40</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4760,21 +4967,21 @@
         <v>8</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="12"/>
+        <v>21</v>
+      </c>
+      <c r="E14" s="13"/>
       <c r="F14" s="9" t="n">
         <f aca="false">2*'통합 청구'!$C$3</f>
         <v>40</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="H14" s="8"/>
     </row>
@@ -4783,24 +4990,24 @@
         <v>9</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E15" s="12"/>
+        <v>24</v>
+      </c>
+      <c r="E15" s="13"/>
       <c r="F15" s="9" t="n">
         <f aca="false">3*'통합 청구'!$C$4</f>
         <v>54</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4808,31 +5015,31 @@
         <v>10</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E16" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E16" s="14" t="n">
         <f aca="false">21250+740+3690</f>
         <v>25680</v>
       </c>
-      <c r="F16" s="13" t="n">
+      <c r="F16" s="14" t="n">
         <v>21000</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
@@ -4847,16 +5054,16 @@
         <v>1</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
+        <v>21</v>
+      </c>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
       <c r="G18" s="8"/>
       <c r="H18" s="8"/>
     </row>
@@ -4865,16 +5072,16 @@
         <v>2</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
+        <v>21</v>
+      </c>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
     </row>
@@ -4883,16 +5090,16 @@
         <v>3</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
+        <v>24</v>
+      </c>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
       <c r="G20" s="8"/>
       <c r="H20" s="8"/>
     </row>
@@ -4901,16 +5108,16 @@
         <v>4</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E21" s="12"/>
-      <c r="F21" s="12"/>
+        <v>24</v>
+      </c>
+      <c r="E21" s="13"/>
+      <c r="F21" s="13"/>
       <c r="G21" s="8"/>
       <c r="H21" s="8"/>
     </row>
@@ -4919,16 +5126,16 @@
         <v>5</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E22" s="12"/>
-      <c r="F22" s="12"/>
+        <v>21</v>
+      </c>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13"/>
       <c r="G22" s="8"/>
       <c r="H22" s="8"/>
     </row>
@@ -4937,16 +5144,16 @@
         <v>6</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E23" s="12"/>
-      <c r="F23" s="12"/>
+        <v>21</v>
+      </c>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
       <c r="G23" s="8"/>
       <c r="H23" s="8"/>
     </row>
@@ -4955,16 +5162,16 @@
         <v>7</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E24" s="12"/>
-      <c r="F24" s="12"/>
+        <v>21</v>
+      </c>
+      <c r="E24" s="13"/>
+      <c r="F24" s="13"/>
       <c r="G24" s="8"/>
       <c r="H24" s="8"/>
     </row>
@@ -4973,16 +5180,16 @@
         <v>8</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12"/>
+        <v>21</v>
+      </c>
+      <c r="E25" s="13"/>
+      <c r="F25" s="13"/>
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
     </row>
@@ -4991,16 +5198,16 @@
         <v>9</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E26" s="12"/>
-      <c r="F26" s="12"/>
+        <v>21</v>
+      </c>
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
       <c r="G26" s="8"/>
       <c r="H26" s="8"/>
     </row>
@@ -5009,19 +5216,19 @@
         <v>10</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E27" s="12"/>
-      <c r="F27" s="12"/>
+        <v>24</v>
+      </c>
+      <c r="E27" s="13"/>
+      <c r="F27" s="13"/>
       <c r="G27" s="8"/>
       <c r="H27" s="8" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5029,19 +5236,19 @@
         <v>11</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E28" s="12"/>
-      <c r="F28" s="12"/>
+        <v>24</v>
+      </c>
+      <c r="E28" s="13"/>
+      <c r="F28" s="13"/>
       <c r="G28" s="8"/>
       <c r="H28" s="8" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5049,19 +5256,19 @@
         <v>12</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E29" s="12"/>
-      <c r="F29" s="12"/>
+        <v>21</v>
+      </c>
+      <c r="E29" s="13"/>
+      <c r="F29" s="13"/>
       <c r="G29" s="8"/>
       <c r="H29" s="8" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5069,16 +5276,16 @@
         <v>13</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E30" s="12"/>
-      <c r="F30" s="12"/>
+        <v>21</v>
+      </c>
+      <c r="E30" s="13"/>
+      <c r="F30" s="13"/>
       <c r="G30" s="8"/>
       <c r="H30" s="8"/>
     </row>
@@ -5087,16 +5294,16 @@
         <v>14</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E31" s="12"/>
-      <c r="F31" s="12"/>
+        <v>21</v>
+      </c>
+      <c r="E31" s="13"/>
+      <c r="F31" s="13"/>
       <c r="G31" s="8"/>
       <c r="H31" s="8"/>
     </row>
@@ -5105,16 +5312,16 @@
         <v>15</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E32" s="12"/>
-      <c r="F32" s="12"/>
+        <v>21</v>
+      </c>
+      <c r="E32" s="13"/>
+      <c r="F32" s="13"/>
       <c r="G32" s="8"/>
       <c r="H32" s="8"/>
     </row>
@@ -5123,16 +5330,16 @@
         <v>16</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E33" s="12"/>
-      <c r="F33" s="12"/>
+        <v>21</v>
+      </c>
+      <c r="E33" s="13"/>
+      <c r="F33" s="13"/>
       <c r="G33" s="8"/>
       <c r="H33" s="8"/>
     </row>
@@ -5141,19 +5348,19 @@
         <v>17</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E34" s="12"/>
-      <c r="F34" s="12"/>
+        <v>24</v>
+      </c>
+      <c r="E34" s="13"/>
+      <c r="F34" s="13"/>
       <c r="G34" s="8"/>
       <c r="H34" s="8" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="47.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5161,16 +5368,16 @@
         <v>18</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E35" s="12"/>
-      <c r="F35" s="12"/>
+        <v>21</v>
+      </c>
+      <c r="E35" s="13"/>
+      <c r="F35" s="13"/>
       <c r="G35" s="8"/>
       <c r="H35" s="8"/>
     </row>
@@ -5179,19 +5386,19 @@
         <v>19</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E36" s="12"/>
-      <c r="F36" s="12"/>
+        <v>21</v>
+      </c>
+      <c r="E36" s="13"/>
+      <c r="F36" s="13"/>
       <c r="G36" s="8"/>
       <c r="H36" s="8" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="36.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5199,19 +5406,19 @@
         <v>20</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E37" s="12"/>
-      <c r="F37" s="12"/>
+        <v>21</v>
+      </c>
+      <c r="E37" s="13"/>
+      <c r="F37" s="13"/>
       <c r="G37" s="8"/>
       <c r="H37" s="8" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5219,16 +5426,16 @@
         <v>21</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E38" s="12"/>
-      <c r="F38" s="12"/>
+        <v>21</v>
+      </c>
+      <c r="E38" s="13"/>
+      <c r="F38" s="13"/>
       <c r="G38" s="8"/>
       <c r="H38" s="8"/>
     </row>
@@ -5266,48 +5473,48 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="11" t="s">
-        <v>120</v>
+      <c r="A2" s="12" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="11" t="s">
-        <v>64</v>
+      <c r="A3" s="12" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="H5" s="5" t="s">
         <v>16</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -5322,20 +5529,20 @@
         <v>1</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C7" s="8"/>
       <c r="D7" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E7" s="14" t="n">
         <v>106</v>
       </c>
-      <c r="F7" s="13" t="n">
+      <c r="F7" s="14" t="n">
         <v>200</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="H7" s="8"/>
     </row>
@@ -5344,20 +5551,20 @@
         <v>2</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C8" s="8"/>
       <c r="D8" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E8" s="14" t="n">
         <v>120</v>
       </c>
-      <c r="F8" s="13" t="n">
+      <c r="F8" s="14" t="n">
         <v>300</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="H8" s="8"/>
     </row>
@@ -5366,20 +5573,20 @@
         <v>3</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C9" s="8"/>
       <c r="D9" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E9" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="13" t="n">
+      <c r="F9" s="14" t="n">
         <v>20</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="H9" s="8"/>
     </row>
@@ -5388,23 +5595,23 @@
         <v>4</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C10" s="8"/>
       <c r="D10" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E10" s="14" t="n">
         <v>25080</v>
       </c>
-      <c r="F10" s="13" t="n">
+      <c r="F10" s="14" t="n">
         <v>30000</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5412,30 +5619,30 @@
         <v>5</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E11" s="14" t="n">
         <v>130</v>
       </c>
-      <c r="F11" s="13" t="n">
+      <c r="F11" s="14" t="n">
         <v>100</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="H11" s="14" t="s">
-        <v>129</v>
+        <v>132</v>
+      </c>
+      <c r="H11" s="11" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
@@ -5445,23 +5652,33 @@
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="15"/>
-      <c r="B13" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="15"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C13" s="8"/>
+      <c r="D13" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <f aca="false">4*'통합 청구'!$C$5</f>
+        <v>75.6</v>
+      </c>
+      <c r="F13" s="13"/>
+      <c r="G13" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="H13" s="11" t="s">
+        <v>136</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A6:H6"/>
     <mergeCell ref="A12:H12"/>
-    <mergeCell ref="B13:H13"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -5492,48 +5709,48 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="11" t="s">
-        <v>133</v>
+      <c r="A2" s="12" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="11" t="s">
-        <v>64</v>
+      <c r="A3" s="12" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="H5" s="5" t="s">
         <v>16</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -5548,20 +5765,20 @@
         <v>1</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="12"/>
-      <c r="F7" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E7" s="13"/>
+      <c r="F7" s="14" t="n">
         <v>120</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="H7" s="8"/>
     </row>
@@ -5570,25 +5787,25 @@
         <v>2</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E8" s="14" t="n">
         <v>27</v>
       </c>
-      <c r="F8" s="13" t="n">
+      <c r="F8" s="14" t="n">
         <v>40</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5596,25 +5813,25 @@
         <v>3</v>
       </c>
       <c r="B9" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="14" t="n">
         <v>27</v>
       </c>
-      <c r="C9" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E9" s="13" t="n">
-        <v>27</v>
-      </c>
-      <c r="F9" s="13" t="n">
+      <c r="F9" s="14" t="n">
         <v>72</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5622,25 +5839,25 @@
         <v>4</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E10" s="13" t="n">
+        <v>24</v>
+      </c>
+      <c r="E10" s="14" t="n">
         <v>52</v>
       </c>
-      <c r="F10" s="13" t="n">
+      <c r="F10" s="14" t="n">
         <v>90</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5648,25 +5865,25 @@
         <v>5</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E11" s="14" t="n">
         <v>48</v>
       </c>
-      <c r="F11" s="13" t="n">
+      <c r="F11" s="14" t="n">
         <v>20</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5674,20 +5891,20 @@
         <v>6</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="12"/>
-      <c r="F12" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E12" s="13"/>
+      <c r="F12" s="14" t="n">
         <v>40</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="H12" s="8"/>
     </row>
@@ -5696,25 +5913,25 @@
         <v>7</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E13" s="14" t="n">
         <v>1400</v>
       </c>
-      <c r="F13" s="13" t="n">
+      <c r="F13" s="14" t="n">
         <v>400</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5722,20 +5939,20 @@
         <v>8</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="12"/>
-      <c r="F14" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E14" s="13"/>
+      <c r="F14" s="14" t="n">
         <v>15000</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="H14" s="8"/>
     </row>
@@ -5744,30 +5961,30 @@
         <v>9</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E15" s="14" t="n">
         <v>70</v>
       </c>
-      <c r="F15" s="13" t="n">
+      <c r="F15" s="14" t="n">
         <v>120</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
@@ -5777,23 +5994,33 @@
       <c r="G16" s="6"/>
       <c r="H16" s="6"/>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="15"/>
-      <c r="B17" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C17" s="8"/>
+      <c r="D17" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E17" s="9" t="n">
+        <f aca="false">5*'통합 청구'!$C$5</f>
+        <v>94.5</v>
+      </c>
+      <c r="F17" s="13"/>
+      <c r="G17" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="H17" s="11" t="s">
+        <v>136</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A6:H6"/>
     <mergeCell ref="A16:H16"/>
-    <mergeCell ref="B17:H17"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -5824,48 +6051,48 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="11" t="s">
-        <v>153</v>
+      <c r="A2" s="12" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="11" t="s">
-        <v>64</v>
+      <c r="A3" s="12" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="H5" s="5" t="s">
         <v>16</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -5880,24 +6107,24 @@
         <v>1</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C7" s="8"/>
       <c r="D7" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7" s="13" t="n">
+        <v>24</v>
+      </c>
+      <c r="E7" s="14" t="n">
         <v>140</v>
       </c>
-      <c r="F7" s="13" t="n">
+      <c r="F7" s="14" t="n">
         <f aca="false">3*18</f>
         <v>54</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5905,24 +6132,24 @@
         <v>2</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C8" s="8"/>
       <c r="D8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E8" s="13" t="n">
+        <v>24</v>
+      </c>
+      <c r="E8" s="14" t="n">
         <v>36</v>
       </c>
-      <c r="F8" s="13" t="n">
+      <c r="F8" s="14" t="n">
         <f aca="false">2*18</f>
         <v>36</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5930,23 +6157,23 @@
         <v>3</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C9" s="8"/>
       <c r="D9" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E9" s="14" t="n">
         <v>130</v>
       </c>
-      <c r="F9" s="13" t="n">
+      <c r="F9" s="14" t="n">
         <v>100</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5954,24 +6181,24 @@
         <v>4</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C10" s="8"/>
       <c r="D10" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E10" s="13" t="n">
+        <v>24</v>
+      </c>
+      <c r="E10" s="14" t="n">
         <v>70</v>
       </c>
-      <c r="F10" s="13" t="n">
+      <c r="F10" s="14" t="n">
         <f aca="false">10*18</f>
         <v>180</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5979,23 +6206,23 @@
         <v>5</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C11" s="8"/>
       <c r="D11" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E11" s="14" t="n">
         <v>40</v>
       </c>
-      <c r="F11" s="13" t="n">
+      <c r="F11" s="14" t="n">
         <v>160</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6003,23 +6230,23 @@
         <v>6</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C12" s="8"/>
       <c r="D12" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E12" s="14" t="n">
         <v>150</v>
       </c>
-      <c r="F12" s="13" t="n">
+      <c r="F12" s="14" t="n">
         <v>100</v>
       </c>
       <c r="G12" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="H12" s="8" t="s">
         <v>162</v>
-      </c>
-      <c r="H12" s="8" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6027,23 +6254,23 @@
         <v>7</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C13" s="8"/>
       <c r="D13" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E13" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="F13" s="13" t="n">
+      <c r="F13" s="14" t="n">
         <v>60</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6051,23 +6278,23 @@
         <v>8</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C14" s="8"/>
       <c r="D14" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E14" s="14" t="n">
         <v>80</v>
       </c>
-      <c r="F14" s="13" t="n">
+      <c r="F14" s="14" t="n">
         <v>60</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6075,23 +6302,23 @@
         <v>9</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C15" s="8"/>
       <c r="D15" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E15" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="F15" s="13" t="n">
+      <c r="F15" s="14" t="n">
         <v>20</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6099,23 +6326,23 @@
         <v>10</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C16" s="8"/>
       <c r="D16" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E16" s="13" t="n">
+        <v>24</v>
+      </c>
+      <c r="E16" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="13" t="n">
+      <c r="F16" s="14" t="n">
         <v>18</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6123,24 +6350,24 @@
         <v>11</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C17" s="8"/>
       <c r="D17" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E17" s="13" t="n">
+        <v>24</v>
+      </c>
+      <c r="E17" s="14" t="n">
         <v>102</v>
       </c>
-      <c r="F17" s="13" t="n">
+      <c r="F17" s="14" t="n">
         <f aca="false">5*18</f>
         <v>90</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6148,24 +6375,24 @@
         <v>12</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C18" s="8"/>
       <c r="D18" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E18" s="13" t="n">
+        <v>24</v>
+      </c>
+      <c r="E18" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="F18" s="13" t="n">
+      <c r="F18" s="14" t="n">
         <f aca="false">0.38*5</f>
         <v>1.9</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6173,20 +6400,20 @@
         <v>13</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C19" s="8"/>
       <c r="D19" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E19" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E19" s="14" t="n">
         <v>19500</v>
       </c>
-      <c r="F19" s="13" t="n">
+      <c r="F19" s="14" t="n">
         <v>45000</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="H19" s="8"/>
     </row>
@@ -6195,31 +6422,31 @@
         <v>14</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E20" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E20" s="14" t="n">
         <v>70</v>
       </c>
-      <c r="F20" s="13" t="n">
+      <c r="F20" s="14" t="n">
         <f aca="false">4*18.9</f>
         <v>75.6</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -6229,23 +6456,33 @@
       <c r="G21" s="6"/>
       <c r="H21" s="6"/>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="15"/>
-      <c r="B22" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="15"/>
-      <c r="F22" s="15"/>
-      <c r="G22" s="15"/>
-      <c r="H22" s="15"/>
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C22" s="8"/>
+      <c r="D22" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E22" s="9" t="n">
+        <f aca="false">5*'통합 청구'!$C$5</f>
+        <v>94.5</v>
+      </c>
+      <c r="F22" s="13"/>
+      <c r="G22" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="H22" s="11" t="s">
+        <v>136</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A6:H6"/>
     <mergeCell ref="A21:H21"/>
-    <mergeCell ref="B22:H22"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>